<commit_message>
add multinomial logistic regression
</commit_message>
<xml_diff>
--- a/docs/resultats.xlsx
+++ b/docs/resultats.xlsx
@@ -37,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -50,6 +50,34 @@
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
     </border>
     <border>
       <left style="thin"/>
@@ -446,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -676,119 +704,194 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>Modalité</t>
+          <t>Catégorie</t>
         </is>
       </c>
       <c r="C23" s="1" t="inlineStr">
         <is>
+          <t>2 - Autant de bien que de mal</t>
+        </is>
+      </c>
+      <c r="D23" s="1" t="n"/>
+      <c r="E23" s="1" t="n"/>
+      <c r="F23" s="1" t="inlineStr">
+        <is>
+          <t>3 - Plus de bien que de mal</t>
+        </is>
+      </c>
+      <c r="G23" s="1" t="n"/>
+      <c r="H23" s="1" t="n"/>
+      <c r="I23" s="1" t="inlineStr">
+        <is>
+          <t>4 - Sans réponse</t>
+        </is>
+      </c>
+      <c r="J23" s="1" t="n"/>
+      <c r="K23" s="1" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="1" t="inlineStr"/>
+      <c r="C24" s="1" t="inlineStr">
+        <is>
           <t>OR</t>
         </is>
       </c>
-      <c r="D23" s="1" t="inlineStr">
+      <c r="D24" s="1" t="inlineStr">
         <is>
           <t>p</t>
         </is>
       </c>
-      <c r="E23" s="1" t="inlineStr">
+      <c r="E24" s="1" t="inlineStr">
         <is>
           <t>IC 95%</t>
         </is>
       </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>.Intercept</t>
-        </is>
-      </c>
-      <c r="B24" s="1" t="inlineStr"/>
-      <c r="C24" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>0.0***</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>0.41 [0.27-0.62]</t>
+      <c r="F24" s="1" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="G24" s="1" t="inlineStr">
+        <is>
+          <t>p</t>
+        </is>
+      </c>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
+          <t>IC 95%</t>
+        </is>
+      </c>
+      <c r="I24" s="1" t="inlineStr">
+        <is>
+          <t>OR</t>
+        </is>
+      </c>
+      <c r="J24" s="1" t="inlineStr">
+        <is>
+          <t>p</t>
+        </is>
+      </c>
+      <c r="K24" s="1" t="inlineStr">
+        <is>
+          <t>IC 95%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="inlineStr">
         <is>
+          <t>Variable</t>
+        </is>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>Modalité</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="inlineStr">
+        <is>
+          <t>.Intercept</t>
+        </is>
+      </c>
+      <c r="B26" s="1" t="inlineStr"/>
+      <c r="C26" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>*** (p &lt; 0.001)</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>7.84 [3.6-17.06]</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>3.81</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>*** (p &lt; 0.001)</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>3.81 [1.69-8.59]</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>(p=0.34)</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>0.51 [0.13-2.05]</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
           <t>Age</t>
         </is>
       </c>
-      <c r="B25" s="1" t="inlineStr">
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>18 à 24 ans</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>ref</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t xml:space="preserve"> </t>
         </is>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="n"/>
-      <c r="B26" s="1" t="inlineStr">
-        <is>
-          <t>25 à 34 ans</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>0.674</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>1.12 [0.67-1.87]</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="n"/>
-      <c r="B27" s="1" t="inlineStr">
-        <is>
-          <t>35 à 49 ans</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>0.197</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>1.36 [0.85-2.17]</t>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>ref</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>ref</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -796,20 +899,46 @@
       <c r="A28" s="1" t="n"/>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>50 à 64 ans</t>
+          <t>25 à 34 ans</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1.73</v>
+        <v>0.68</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>0.021*</t>
+          <t>(p=0.39)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.73 [1.09-2.77]</t>
+          <t>0.68 [0.28-1.65]</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>0.77</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>(p=0.58)</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>0.77 [0.31-1.94]</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>(p=0.17)</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>0.25 [0.04-1.81]</t>
         </is>
       </c>
     </row>
@@ -817,47 +946,93 @@
       <c r="A29" s="1" t="n"/>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>65 ans et+</t>
+          <t>35 à 49 ans</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1.74</v>
+        <v>1.3</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>0.023*</t>
+          <t>(p=0.57)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.74 [1.08-2.79]</t>
+          <t>1.3 [0.53-3.21]</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>(p=0.36)</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>1.55 [0.61-3.96]</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>(p=0.62)</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>0.65 [0.12-3.63]</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="inlineStr">
-        <is>
-          <t>Genre</t>
-        </is>
-      </c>
+      <c r="A30" s="1" t="n"/>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>Femme</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>ref</t>
-        </is>
+          <t>50 à 64 ans</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>1.25</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>(p=0.63)</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> </t>
+          <t>1.25 [0.5-3.16]</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>(p=0.15)</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2.03 [0.78-5.25]</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>(p=0.39)</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>0.42 [0.06-3.05]</t>
         </is>
       </c>
     </row>
@@ -865,27 +1040,160 @@
       <c r="A31" s="1" t="n"/>
       <c r="B31" s="1" t="inlineStr">
         <is>
+          <t>65 ans et+</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>(p=0.28)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1.77 [0.63-4.97]</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>2.81</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>(p=0.06)</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2.81 [0.97-8.09]</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>(p=0.94)</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>1.07 [0.16-7.04]</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr">
+        <is>
+          <t>Genre</t>
+        </is>
+      </c>
+      <c r="B32" s="1" t="inlineStr">
+        <is>
+          <t>Femme</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>ref</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>ref</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>ref</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n"/>
+      <c r="B33" s="1" t="inlineStr">
+        <is>
           <t>Homme</t>
         </is>
       </c>
-      <c r="C31" t="n">
-        <v>1.41</v>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>0.007**</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>1.41 [1.10-1.82]</t>
+      <c r="C33" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>(p=0.51)</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>0.84 [0.5-1.41]</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>(p=0.55)</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>1.18 [0.69-2.0]</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>(p=0.19)</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>0.43 [0.12-1.52]</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A25:A29"/>
-    <mergeCell ref="A30:A31"/>
+  <mergeCells count="5">
+    <mergeCell ref="F23:H23"/>
+    <mergeCell ref="A32:A33"/>
+    <mergeCell ref="A27:A31"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="I23:K23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>